<commit_message>
new tabular dataset constructed
</commit_message>
<xml_diff>
--- a/dataset/construct/dataset_splits/data_size/10_percent/lmu/fold1.xlsx
+++ b/dataset/construct/dataset_splits/data_size/10_percent/lmu/fold1.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AN15"/>
+  <dimension ref="A1:AK15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,185 +446,170 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>DM</t>
+          <t>BMI</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>BMI</t>
+          <t>AFPRE</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>CABGPRE</t>
+          <t>LVEFPRE</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>AFPRE</t>
+          <t>PREDILATION</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>LVEFPRE</t>
+          <t>CT_ValScNCC</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>NTPROBNPPRE</t>
+          <t>CT_ValScRCC</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>PREDILATION</t>
+          <t>CT_ValScLCC</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>CT_ValScNCC</t>
+          <t>CT_ValvScTot</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>CT_ValScRCC</t>
+          <t>CT_AnnScNCC</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>CT_ValScLCC</t>
+          <t>CT_AnnScRCC</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>CT_ValvScTot</t>
+          <t>CT_AnnScLCC</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>CT_AnnScNCC</t>
+          <t>CT_AnnScTot</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>CT_AnnScRCC</t>
+          <t>CT_LVOTScNCC</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>CT_AnnScLCC</t>
+          <t>CT_LVOTScRCC</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>CT_AnnScTot</t>
+          <t>CT_LVOTScLCC</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>CT_LVOTScNCC</t>
+          <t>CT_LVOTScTot</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>CT_LVOTScRCC</t>
+          <t>SEX</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>CT_LVOTScLCC</t>
+          <t>CT_AnnMean</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>CT_LVOTScTot</t>
+          <t>ECC_INDEX</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>SEX</t>
+          <t>CT_Peri_Deri</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>CT_AnnMean</t>
+          <t>CT_Area_Deri</t>
         </is>
       </c>
       <c r="Y1" s="1" t="inlineStr">
         <is>
-          <t>ECC_INDEX</t>
+          <t>nyha2</t>
         </is>
       </c>
       <c r="Z1" s="1" t="inlineStr">
         <is>
-          <t>CT_Peri_Deri</t>
+          <t>nyha3</t>
         </is>
       </c>
       <c r="AA1" s="1" t="inlineStr">
         <is>
-          <t>CT_Area_Deri</t>
+          <t>nyha4</t>
         </is>
       </c>
       <c r="AB1" s="1" t="inlineStr">
         <is>
-          <t>nyha2</t>
+          <t>model1</t>
         </is>
       </c>
       <c r="AC1" s="1" t="inlineStr">
         <is>
-          <t>nyha3</t>
+          <t>model2</t>
         </is>
       </c>
       <c r="AD1" s="1" t="inlineStr">
         <is>
-          <t>nyha4</t>
+          <t>model3</t>
         </is>
       </c>
       <c r="AE1" s="1" t="inlineStr">
         <is>
-          <t>model1</t>
+          <t>model4</t>
         </is>
       </c>
       <c r="AF1" s="1" t="inlineStr">
         <is>
-          <t>model2</t>
+          <t>model7</t>
         </is>
       </c>
       <c r="AG1" s="1" t="inlineStr">
         <is>
-          <t>model3</t>
+          <t>model8</t>
         </is>
       </c>
       <c r="AH1" s="1" t="inlineStr">
         <is>
-          <t>model4</t>
+          <t>brand2</t>
         </is>
       </c>
       <c r="AI1" s="1" t="inlineStr">
         <is>
-          <t>model7</t>
+          <t>brand8</t>
         </is>
       </c>
       <c r="AJ1" s="1" t="inlineStr">
         <is>
-          <t>model8</t>
+          <t>QRSADM</t>
         </is>
       </c>
       <c r="AK1" s="1" t="inlineStr">
-        <is>
-          <t>brand2</t>
-        </is>
-      </c>
-      <c r="AL1" s="1" t="inlineStr">
-        <is>
-          <t>brand8</t>
-        </is>
-      </c>
-      <c r="AM1" s="1" t="inlineStr">
-        <is>
-          <t>QRSADM</t>
-        </is>
-      </c>
-      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>PQADM</t>
         </is>
@@ -632,7 +617,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>54822613</v>
+        <v>54380016</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -640,74 +625,80 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>64.34496919917861</v>
-      </c>
-      <c r="D2" t="inlineStr"/>
+        <v>82.3299110198494</v>
+      </c>
+      <c r="D2" t="n">
+        <v>33.2179930795848</v>
+      </c>
       <c r="E2" t="n">
-        <v>34.6666666666667</v>
-      </c>
-      <c r="F2" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="F2" t="n">
+        <v>45</v>
+      </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
-      <c r="H2" t="n">
-        <v>50</v>
-      </c>
+      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr"/>
-      <c r="J2" t="n">
-        <v>1</v>
-      </c>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
+      <c r="L2" t="n">
+        <v>419</v>
+      </c>
+      <c r="M2" t="n">
+        <v>133</v>
+      </c>
+      <c r="N2" t="n">
+        <v>100</v>
+      </c>
       <c r="O2" t="n">
-        <v>251</v>
+        <v>652</v>
       </c>
       <c r="P2" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>72</v>
+        <v>0</v>
       </c>
       <c r="R2" t="n">
-        <v>343</v>
+        <v>69</v>
       </c>
       <c r="S2" t="n">
-        <v>0</v>
+        <v>69</v>
       </c>
       <c r="T2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U2" t="n">
-        <v>41</v>
+        <v>25.1</v>
       </c>
       <c r="V2" t="n">
-        <v>41</v>
+        <v>0.23</v>
       </c>
       <c r="W2" t="n">
-        <v>2</v>
+        <v>25.14648100851947</v>
       </c>
       <c r="X2" t="n">
-        <v>20</v>
+        <v>24.59245379682967</v>
       </c>
       <c r="Y2" t="n">
-        <v>0.23</v>
+        <v>0</v>
       </c>
       <c r="Z2" t="n">
-        <v>63.9</v>
+        <v>1</v>
       </c>
       <c r="AA2" t="n">
-        <v>314.2</v>
+        <v>0</v>
       </c>
       <c r="AB2" t="n">
         <v>0</v>
       </c>
       <c r="AC2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE2" t="n">
         <v>0</v>
@@ -716,33 +707,24 @@
         <v>0</v>
       </c>
       <c r="AG2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AH2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" t="n">
-        <v>0</v>
+        <v>191</v>
       </c>
       <c r="AK2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM2" t="n">
-        <v>174</v>
-      </c>
-      <c r="AN2" t="n">
-        <v>99</v>
+        <v>132</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>53731161</v>
+        <v>51310921</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -750,74 +732,88 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>87.4661190965092</v>
-      </c>
-      <c r="D3" t="inlineStr"/>
+        <v>82.76796714579049</v>
+      </c>
+      <c r="D3" t="n">
+        <v>23.8086901719128</v>
+      </c>
       <c r="E3" t="n">
-        <v>24.3374797187669</v>
-      </c>
-      <c r="F3" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>50</v>
+      </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H3" t="n">
-        <v>55</v>
-      </c>
-      <c r="I3" t="inlineStr"/>
+        <v>414</v>
+      </c>
+      <c r="I3" t="n">
+        <v>322</v>
+      </c>
       <c r="J3" t="n">
-        <v>1</v>
-      </c>
-      <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
+        <v>250</v>
+      </c>
+      <c r="K3" t="n">
+        <v>986</v>
+      </c>
+      <c r="L3" t="n">
+        <v>414</v>
+      </c>
+      <c r="M3" t="n">
+        <v>322</v>
+      </c>
+      <c r="N3" t="n">
+        <v>221</v>
+      </c>
       <c r="O3" t="n">
-        <v>489.90607</v>
+        <v>957</v>
       </c>
       <c r="P3" t="n">
-        <v>244.57335</v>
+        <v>43</v>
       </c>
       <c r="Q3" t="n">
-        <v>201.23125</v>
+        <v>0</v>
       </c>
       <c r="R3" t="n">
-        <v>935.71075</v>
+        <v>225</v>
       </c>
       <c r="S3" t="n">
-        <v>229</v>
+        <v>268</v>
       </c>
       <c r="T3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U3" t="n">
-        <v>35</v>
+        <v>27.6</v>
       </c>
       <c r="V3" t="n">
-        <v>263</v>
+        <v>0.14</v>
       </c>
       <c r="W3" t="n">
-        <v>1</v>
+        <v>28.52056580206764</v>
       </c>
       <c r="X3" t="n">
-        <v>24.043266</v>
+        <v>27.79113361913022</v>
       </c>
       <c r="Y3" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="Z3" t="n">
-        <v>78.1448</v>
+        <v>1</v>
       </c>
       <c r="AA3" t="n">
-        <v>470.0287</v>
+        <v>0</v>
       </c>
       <c r="AB3" t="n">
         <v>0</v>
       </c>
       <c r="AC3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE3" t="n">
         <v>0</v>
@@ -835,20 +831,15 @@
         <v>0</v>
       </c>
       <c r="AJ3" t="n">
-        <v>0</v>
+        <v>192</v>
       </c>
       <c r="AK3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM3" t="inlineStr"/>
-      <c r="AN3" t="inlineStr"/>
+        <v>182</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>53291409</v>
+        <v>53146249</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -856,84 +847,88 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>81.79329226557149</v>
+        <v>74.03969883641339</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>29.0687961508904</v>
       </c>
       <c r="E4" t="n">
-        <v>28</v>
-      </c>
-      <c r="F4" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>45</v>
+      </c>
       <c r="G4" t="n">
         <v>1</v>
       </c>
       <c r="H4" t="n">
-        <v>55</v>
-      </c>
-      <c r="I4" t="inlineStr"/>
+        <v>1326</v>
+      </c>
+      <c r="I4" t="n">
+        <v>773</v>
+      </c>
       <c r="J4" t="n">
-        <v>1</v>
+        <v>426</v>
       </c>
       <c r="K4" t="n">
-        <v>310</v>
+        <v>2525</v>
       </c>
       <c r="L4" t="n">
-        <v>66</v>
+        <v>1320</v>
       </c>
       <c r="M4" t="n">
-        <v>63</v>
+        <v>718</v>
       </c>
       <c r="N4" t="n">
-        <v>439</v>
+        <v>384</v>
       </c>
       <c r="O4" t="n">
-        <v>310</v>
+        <v>2422</v>
       </c>
       <c r="P4" t="n">
-        <v>60</v>
+        <v>96</v>
       </c>
       <c r="Q4" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="R4" t="n">
-        <v>425</v>
+        <v>61</v>
       </c>
       <c r="S4" t="n">
-        <v>0</v>
+        <v>157</v>
       </c>
       <c r="T4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U4" t="n">
-        <v>0</v>
+        <v>25.2</v>
       </c>
       <c r="V4" t="n">
-        <v>0</v>
+        <v>0.39</v>
       </c>
       <c r="W4" t="n">
-        <v>2</v>
+        <v>26.03774868983408</v>
       </c>
       <c r="X4" t="n">
-        <v>23.1</v>
+        <v>24.58986498122201</v>
       </c>
       <c r="Y4" t="n">
-        <v>0.34</v>
+        <v>0</v>
       </c>
       <c r="Z4" t="n">
-        <v>74.09999999999999</v>
+        <v>1</v>
       </c>
       <c r="AA4" t="n">
-        <v>397</v>
+        <v>0</v>
       </c>
       <c r="AB4" t="n">
         <v>0</v>
       </c>
       <c r="AC4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE4" t="n">
         <v>0</v>
@@ -945,26 +940,21 @@
         <v>0</v>
       </c>
       <c r="AH4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ4" t="n">
-        <v>0</v>
+        <v>148</v>
       </c>
       <c r="AK4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM4" t="inlineStr"/>
-      <c r="AN4" t="inlineStr"/>
+        <v>109</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>54786923</v>
+        <v>54397745</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -972,74 +962,80 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>74.4284736481862</v>
-      </c>
-      <c r="D5" t="inlineStr"/>
+        <v>91.668720054757</v>
+      </c>
+      <c r="D5" t="n">
+        <v>25.2173585757838</v>
+      </c>
       <c r="E5" t="n">
-        <v>25.013520822066</v>
-      </c>
-      <c r="F5" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>60</v>
+      </c>
       <c r="G5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" t="n">
-        <v>60</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
-      <c r="J5" t="n">
-        <v>1</v>
-      </c>
+      <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
+      <c r="L5" t="n">
+        <v>252</v>
+      </c>
+      <c r="M5" t="n">
+        <v>110</v>
+      </c>
+      <c r="N5" t="n">
+        <v>324</v>
+      </c>
       <c r="O5" t="n">
-        <v>115</v>
+        <v>686</v>
       </c>
       <c r="P5" t="n">
-        <v>188</v>
+        <v>420</v>
       </c>
       <c r="Q5" t="n">
-        <v>170</v>
+        <v>50</v>
       </c>
       <c r="R5" t="n">
-        <v>474</v>
+        <v>202</v>
       </c>
       <c r="S5" t="n">
-        <v>0</v>
+        <v>672</v>
       </c>
       <c r="T5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U5" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="V5" t="n">
-        <v>0</v>
+        <v>0.33</v>
       </c>
       <c r="W5" t="n">
-        <v>1</v>
+        <v>22.72732587352266</v>
       </c>
       <c r="X5" t="n">
-        <v>25.6</v>
+        <v>21.03753944143522</v>
       </c>
       <c r="Y5" t="n">
-        <v>0.27</v>
+        <v>0</v>
       </c>
       <c r="Z5" t="n">
-        <v>86.40000000000001</v>
+        <v>1</v>
       </c>
       <c r="AA5" t="n">
-        <v>535.8</v>
+        <v>0</v>
       </c>
       <c r="AB5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AC5" t="n">
         <v>0</v>
       </c>
       <c r="AD5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE5" t="n">
         <v>0</v>
@@ -1051,30 +1047,21 @@
         <v>0</v>
       </c>
       <c r="AH5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AI5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ5" t="n">
-        <v>0</v>
+        <v>104</v>
       </c>
       <c r="AK5" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM5" t="n">
-        <v>118</v>
-      </c>
-      <c r="AN5" t="n">
-        <v>174</v>
+        <v>189</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>53683397</v>
+        <v>53324217</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -1082,84 +1069,88 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>82.2149212867899</v>
+        <v>78.8227241615332</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>25.3515413737155</v>
       </c>
       <c r="E6" t="n">
-        <v>27.0538027739674</v>
-      </c>
-      <c r="F6" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="F6" t="n">
+        <v>50</v>
+      </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>55</v>
-      </c>
-      <c r="I6" t="inlineStr"/>
+        <v>284</v>
+      </c>
+      <c r="I6" t="n">
+        <v>215</v>
+      </c>
       <c r="J6" t="n">
-        <v>1</v>
+        <v>167</v>
       </c>
       <c r="K6" t="n">
-        <v>457</v>
+        <v>666</v>
       </c>
       <c r="L6" t="n">
-        <v>187</v>
+        <v>284</v>
       </c>
       <c r="M6" t="n">
-        <v>138</v>
+        <v>42</v>
       </c>
       <c r="N6" t="n">
-        <v>781</v>
+        <v>93</v>
       </c>
       <c r="O6" t="n">
-        <v>457</v>
+        <v>419</v>
       </c>
       <c r="P6" t="n">
-        <v>187</v>
+        <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>138</v>
+        <v>0</v>
       </c>
       <c r="R6" t="n">
-        <v>781</v>
+        <v>0</v>
       </c>
       <c r="S6" t="n">
         <v>0</v>
       </c>
       <c r="T6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U6" t="n">
-        <v>0</v>
+        <v>26.9</v>
       </c>
       <c r="V6" t="n">
-        <v>0</v>
+        <v>0.28</v>
       </c>
       <c r="W6" t="n">
-        <v>2</v>
+        <v>27.02450933700383</v>
       </c>
       <c r="X6" t="n">
-        <v>24.1</v>
+        <v>25.9134431500973</v>
       </c>
       <c r="Y6" t="n">
-        <v>0.35</v>
+        <v>0</v>
       </c>
       <c r="Z6" t="n">
-        <v>79.8</v>
+        <v>1</v>
       </c>
       <c r="AA6" t="n">
-        <v>463.9</v>
+        <v>0</v>
       </c>
       <c r="AB6" t="n">
         <v>0</v>
       </c>
       <c r="AC6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE6" t="n">
         <v>0</v>
@@ -1168,33 +1159,24 @@
         <v>0</v>
       </c>
       <c r="AG6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AH6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI6" t="n">
         <v>0</v>
       </c>
       <c r="AJ6" t="n">
-        <v>0</v>
+        <v>156</v>
       </c>
       <c r="AK6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL6" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM6" t="n">
-        <v>159</v>
-      </c>
-      <c r="AN6" t="n">
-        <v>130</v>
+        <v>113</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>53940332</v>
+        <v>53688310</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -1202,71 +1184,85 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>89.42915811088299</v>
-      </c>
-      <c r="D7" t="inlineStr"/>
+        <v>92.7775496235455</v>
+      </c>
+      <c r="D7" t="n">
+        <v>30.4498269896194</v>
+      </c>
       <c r="E7" t="n">
-        <v>24.2214532871972</v>
-      </c>
-      <c r="F7" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="F7" t="n">
+        <v>50</v>
+      </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H7" t="n">
-        <v>60</v>
-      </c>
-      <c r="I7" t="inlineStr"/>
+        <v>683</v>
+      </c>
+      <c r="I7" t="n">
+        <v>643</v>
+      </c>
       <c r="J7" t="n">
-        <v>1</v>
-      </c>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
+        <v>414</v>
+      </c>
+      <c r="K7" t="n">
+        <v>1740</v>
+      </c>
+      <c r="L7" t="n">
+        <v>683</v>
+      </c>
+      <c r="M7" t="n">
+        <v>574</v>
+      </c>
+      <c r="N7" t="n">
+        <v>408</v>
+      </c>
       <c r="O7" t="n">
-        <v>116</v>
+        <v>1665</v>
       </c>
       <c r="P7" t="n">
-        <v>215</v>
+        <v>20</v>
       </c>
       <c r="Q7" t="n">
-        <v>98</v>
+        <v>0</v>
       </c>
       <c r="R7" t="n">
-        <v>428</v>
+        <v>11</v>
       </c>
       <c r="S7" t="n">
-        <v>9</v>
+        <v>31</v>
       </c>
       <c r="T7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U7" t="n">
-        <v>0</v>
+        <v>26.5</v>
       </c>
       <c r="V7" t="n">
-        <v>9</v>
+        <v>0.19</v>
       </c>
       <c r="W7" t="n">
-        <v>1</v>
+        <v>26.57887549634652</v>
       </c>
       <c r="X7" t="n">
-        <v>21.4</v>
+        <v>26.20416162512499</v>
       </c>
       <c r="Y7" t="n">
-        <v>0.24</v>
+        <v>0</v>
       </c>
       <c r="Z7" t="n">
-        <v>71</v>
+        <v>0</v>
       </c>
       <c r="AA7" t="n">
-        <v>380.1</v>
+        <v>1</v>
       </c>
       <c r="AB7" t="n">
         <v>0</v>
       </c>
       <c r="AC7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD7" t="n">
         <v>0</v>
@@ -1275,7 +1271,7 @@
         <v>0</v>
       </c>
       <c r="AF7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AG7" t="n">
         <v>0</v>
@@ -1284,27 +1280,14 @@
         <v>0</v>
       </c>
       <c r="AI7" t="n">
-        <v>1</v>
-      </c>
-      <c r="AJ7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM7" t="n">
-        <v>134</v>
-      </c>
-      <c r="AN7" t="n">
-        <v>128</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AJ7" t="inlineStr"/>
+      <c r="AK7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>53592996</v>
+        <v>53959319</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -1312,84 +1295,80 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>81.8617385352498</v>
+        <v>82.8637919233402</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>24.7251829329413</v>
       </c>
       <c r="E8" t="n">
-        <v>27.4692816635161</v>
-      </c>
-      <c r="F8" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>55</v>
+      </c>
       <c r="G8" t="n">
         <v>0</v>
       </c>
-      <c r="H8" t="n">
-        <v>37</v>
-      </c>
+      <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
-      <c r="J8" t="n">
-        <v>1</v>
-      </c>
-      <c r="K8" t="n">
-        <v>1122</v>
-      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
       <c r="L8" t="n">
-        <v>512</v>
+        <v>331</v>
       </c>
       <c r="M8" t="n">
-        <v>1058</v>
+        <v>197</v>
       </c>
       <c r="N8" t="n">
-        <v>2692</v>
+        <v>113</v>
       </c>
       <c r="O8" t="n">
-        <v>1043</v>
+        <v>641</v>
       </c>
       <c r="P8" t="n">
-        <v>506</v>
+        <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>1058</v>
+        <v>0</v>
       </c>
       <c r="R8" t="n">
-        <v>2608</v>
+        <v>0</v>
       </c>
       <c r="S8" t="n">
         <v>0</v>
       </c>
       <c r="T8" t="n">
-        <v>45</v>
+        <v>1</v>
       </c>
       <c r="U8" t="n">
-        <v>307</v>
+        <v>24.1</v>
       </c>
       <c r="V8" t="n">
-        <v>352</v>
+        <v>0.3</v>
       </c>
       <c r="W8" t="n">
-        <v>1</v>
+        <v>25.4011289174665</v>
       </c>
       <c r="X8" t="n">
-        <v>31.5</v>
+        <v>24.50428063210799</v>
       </c>
       <c r="Y8" t="n">
-        <v>0.21</v>
+        <v>1</v>
       </c>
       <c r="Z8" t="n">
-        <v>105.9</v>
+        <v>0</v>
       </c>
       <c r="AA8" t="n">
-        <v>827</v>
+        <v>0</v>
       </c>
       <c r="AB8" t="n">
         <v>0</v>
       </c>
       <c r="AC8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE8" t="n">
         <v>0</v>
@@ -1407,24 +1386,15 @@
         <v>0</v>
       </c>
       <c r="AJ8" t="n">
-        <v>0</v>
+        <v>145</v>
       </c>
       <c r="AK8" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM8" t="n">
-        <v>186</v>
-      </c>
-      <c r="AN8" t="n">
-        <v>109</v>
+        <v>148</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>54742613</v>
+        <v>54859265</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -1432,109 +1402,106 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>72.1587953456537</v>
-      </c>
-      <c r="D9" t="inlineStr"/>
+        <v>70.1054072553046</v>
+      </c>
+      <c r="D9" t="n">
+        <v>29.9616116850286</v>
+      </c>
       <c r="E9" t="n">
-        <v>30.8979120501857</v>
-      </c>
-      <c r="F9" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>55</v>
+      </c>
       <c r="G9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" t="n">
-        <v>47</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
-      <c r="J9" t="n">
-        <v>0</v>
-      </c>
+      <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
+      <c r="L9" t="n">
+        <v>626</v>
+      </c>
+      <c r="M9" t="n">
+        <v>315</v>
+      </c>
+      <c r="N9" t="n">
+        <v>291</v>
+      </c>
       <c r="O9" t="n">
-        <v>203</v>
+        <v>1232</v>
       </c>
       <c r="P9" t="n">
-        <v>109</v>
+        <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>215</v>
+        <v>0</v>
       </c>
       <c r="R9" t="n">
-        <v>527</v>
+        <v>0</v>
       </c>
       <c r="S9" t="n">
         <v>0</v>
       </c>
       <c r="T9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U9" t="n">
-        <v>0</v>
+        <v>26.5</v>
       </c>
       <c r="V9" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="W9" t="n">
-        <v>1</v>
+        <v>27.47014317766114</v>
       </c>
       <c r="X9" t="n">
-        <v>25.5</v>
+        <v>26.53730943771464</v>
       </c>
       <c r="Y9" t="n">
-        <v>0.21</v>
+        <v>0</v>
       </c>
       <c r="Z9" t="n">
-        <v>80.5</v>
+        <v>1</v>
       </c>
       <c r="AA9" t="n">
-        <v>498.6</v>
+        <v>0</v>
       </c>
       <c r="AB9" t="n">
         <v>0</v>
       </c>
       <c r="AC9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD9" t="n">
         <v>0</v>
       </c>
       <c r="AE9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF9" t="n">
         <v>0</v>
       </c>
       <c r="AG9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AH9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI9" t="n">
         <v>0</v>
       </c>
       <c r="AJ9" t="n">
-        <v>0</v>
+        <v>182</v>
       </c>
       <c r="AK9" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL9" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM9" t="n">
-        <v>177</v>
-      </c>
-      <c r="AN9" t="n">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>52530187</v>
+        <v>52386464</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -1542,121 +1509,114 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>78.5516769336071</v>
+        <v>82.11909650924029</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>24.3827160493827</v>
       </c>
       <c r="E10" t="n">
-        <v>27.9296875</v>
+        <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="G10" t="n">
         <v>1</v>
       </c>
       <c r="H10" t="n">
-        <v>55</v>
-      </c>
-      <c r="I10" t="inlineStr"/>
+        <v>257</v>
+      </c>
+      <c r="I10" t="n">
+        <v>546</v>
+      </c>
       <c r="J10" t="n">
-        <v>1</v>
+        <v>368</v>
       </c>
       <c r="K10" t="n">
-        <v>96</v>
+        <v>1171</v>
       </c>
       <c r="L10" t="n">
-        <v>79</v>
+        <v>243</v>
       </c>
       <c r="M10" t="n">
-        <v>258</v>
+        <v>540</v>
       </c>
       <c r="N10" t="n">
-        <v>433</v>
+        <v>368</v>
       </c>
       <c r="O10" t="n">
-        <v>72</v>
+        <v>1151</v>
       </c>
       <c r="P10" t="n">
-        <v>41</v>
+        <v>17</v>
       </c>
       <c r="Q10" t="n">
-        <v>58</v>
+        <v>0</v>
       </c>
       <c r="R10" t="n">
-        <v>171</v>
+        <v>18</v>
       </c>
       <c r="S10" t="n">
-        <v>136</v>
+        <v>35</v>
       </c>
       <c r="T10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U10" t="n">
-        <v>19</v>
+        <v>30.6</v>
       </c>
       <c r="V10" t="n">
-        <v>155</v>
+        <v>0.23</v>
       </c>
       <c r="W10" t="n">
-        <v>2</v>
+        <v>31.73549565252393</v>
       </c>
       <c r="X10" t="n">
-        <v>24.5</v>
+        <v>31.00887782851864</v>
       </c>
       <c r="Y10" t="n">
-        <v>0.33</v>
+        <v>0</v>
       </c>
       <c r="Z10" t="n">
-        <v>78.2</v>
+        <v>1</v>
       </c>
       <c r="AA10" t="n">
-        <v>442.7</v>
+        <v>0</v>
       </c>
       <c r="AB10" t="n">
         <v>0</v>
       </c>
       <c r="AC10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD10" t="n">
         <v>0</v>
       </c>
       <c r="AE10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AG10" t="n">
         <v>0</v>
       </c>
       <c r="AH10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI10" t="n">
         <v>0</v>
       </c>
       <c r="AJ10" t="n">
-        <v>0</v>
+        <v>262</v>
       </c>
       <c r="AK10" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM10" t="n">
-        <v>194</v>
-      </c>
-      <c r="AN10" t="n">
-        <v>126</v>
+        <v>186</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>51748563</v>
+        <v>54879462</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -1664,121 +1624,106 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>80.46269678302529</v>
+        <v>81.138945927447</v>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>32.4499729583559</v>
       </c>
       <c r="E11" t="n">
-        <v>25.390625</v>
+        <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>1</v>
+        <v>55</v>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" t="n">
-        <v>50</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
-      <c r="J11" t="n">
-        <v>1</v>
-      </c>
-      <c r="K11" t="n">
-        <v>47</v>
-      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
       <c r="L11" t="n">
-        <v>432</v>
+        <v>463</v>
       </c>
       <c r="M11" t="n">
-        <v>266</v>
+        <v>138</v>
       </c>
       <c r="N11" t="n">
-        <v>744</v>
+        <v>534</v>
       </c>
       <c r="O11" t="n">
-        <v>47</v>
+        <v>1135</v>
       </c>
       <c r="P11" t="n">
-        <v>302</v>
+        <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>210</v>
+        <v>0</v>
       </c>
       <c r="R11" t="n">
-        <v>559</v>
+        <v>0</v>
       </c>
       <c r="S11" t="n">
         <v>0</v>
       </c>
       <c r="T11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U11" t="n">
-        <v>0</v>
+        <v>25.4</v>
       </c>
       <c r="V11" t="n">
-        <v>0</v>
+        <v>0.26</v>
       </c>
       <c r="W11" t="n">
-        <v>1</v>
+        <v>27.18366428009573</v>
       </c>
       <c r="X11" t="n">
-        <v>24.8</v>
+        <v>26.14091933462482</v>
       </c>
       <c r="Y11" t="n">
-        <v>0.21</v>
+        <v>1</v>
       </c>
       <c r="Z11" t="n">
-        <v>78.3</v>
+        <v>0</v>
       </c>
       <c r="AA11" t="n">
-        <v>461.6</v>
+        <v>0</v>
       </c>
       <c r="AB11" t="n">
         <v>0</v>
       </c>
       <c r="AC11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD11" t="n">
         <v>0</v>
       </c>
       <c r="AE11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF11" t="n">
         <v>0</v>
       </c>
       <c r="AG11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AH11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI11" t="n">
         <v>0</v>
       </c>
       <c r="AJ11" t="n">
-        <v>0</v>
+        <v>224</v>
       </c>
       <c r="AK11" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM11" t="n">
-        <v>120</v>
-      </c>
-      <c r="AN11" t="n">
-        <v>198</v>
+        <v>132</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>51721443</v>
+        <v>52588750</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -1786,119 +1731,114 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>83.8685831622177</v>
+        <v>75.9260780287474</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>24.6913580246914</v>
       </c>
       <c r="E12" t="n">
-        <v>26.4721074380165</v>
+        <v>1</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="G12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H12" t="n">
+        <v>552</v>
+      </c>
+      <c r="I12" t="n">
+        <v>563</v>
+      </c>
       <c r="J12" t="n">
-        <v>1</v>
+        <v>425</v>
       </c>
       <c r="K12" t="n">
-        <v>910</v>
+        <v>1540</v>
       </c>
       <c r="L12" t="n">
-        <v>581</v>
+        <v>531</v>
       </c>
       <c r="M12" t="n">
-        <v>808</v>
+        <v>496</v>
       </c>
       <c r="N12" t="n">
-        <v>2298</v>
+        <v>425</v>
       </c>
       <c r="O12" t="n">
-        <v>910</v>
+        <v>1452</v>
       </c>
       <c r="P12" t="n">
-        <v>431</v>
+        <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>677</v>
+        <v>0</v>
       </c>
       <c r="R12" t="n">
-        <v>2018</v>
+        <v>0</v>
       </c>
       <c r="S12" t="n">
         <v>0</v>
       </c>
       <c r="T12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U12" t="n">
-        <v>0</v>
+        <v>30.4</v>
       </c>
       <c r="V12" t="n">
-        <v>0</v>
+        <v>0.32</v>
       </c>
       <c r="W12" t="n">
-        <v>1</v>
+        <v>31.86281960699744</v>
       </c>
       <c r="X12" t="n">
-        <v>29.5</v>
+        <v>30.32801093241496</v>
       </c>
       <c r="Y12" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="Z12" t="n">
-        <v>93.5</v>
+        <v>0</v>
       </c>
       <c r="AA12" t="n">
-        <v>647.7</v>
+        <v>1</v>
       </c>
       <c r="AB12" t="n">
         <v>0</v>
       </c>
       <c r="AC12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD12" t="n">
         <v>0</v>
       </c>
       <c r="AE12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF12" t="n">
         <v>0</v>
       </c>
       <c r="AG12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AH12" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI12" t="n">
         <v>0</v>
       </c>
       <c r="AJ12" t="n">
-        <v>0</v>
+        <v>174</v>
       </c>
       <c r="AK12" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL12" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM12" t="n">
-        <v>124</v>
-      </c>
-      <c r="AN12" t="n">
-        <v>150</v>
+        <v>211</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>54153818</v>
+        <v>51437724</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
@@ -1906,65 +1846,69 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>79.7891854893908</v>
-      </c>
-      <c r="D13" t="inlineStr"/>
+        <v>89.8179329226557</v>
+      </c>
+      <c r="D13" t="n">
+        <v>17.8359096313912</v>
+      </c>
       <c r="E13" t="n">
-        <v>32.6293520742945</v>
+        <v>1</v>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" t="n">
-        <v>66</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
-      <c r="J13" t="n">
-        <v>0</v>
-      </c>
+      <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
+      <c r="L13" t="n">
+        <v>245.42831</v>
+      </c>
+      <c r="M13" t="n">
+        <v>174.54457</v>
+      </c>
+      <c r="N13" t="n">
+        <v>138.30325</v>
+      </c>
       <c r="O13" t="n">
-        <v>175</v>
+        <v>558.27613</v>
       </c>
       <c r="P13" t="n">
-        <v>213</v>
+        <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>116</v>
+        <v>0</v>
       </c>
       <c r="R13" t="n">
-        <v>505</v>
+        <v>0</v>
       </c>
       <c r="S13" t="n">
         <v>0</v>
       </c>
       <c r="T13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U13" t="n">
-        <v>0</v>
+        <v>24.227337</v>
       </c>
       <c r="V13" t="n">
-        <v>0</v>
+        <v>0.24</v>
       </c>
       <c r="W13" t="n">
-        <v>1</v>
+        <v>24.40130674242708</v>
       </c>
       <c r="X13" t="n">
-        <v>23.6</v>
+        <v>23.98987581932773</v>
       </c>
       <c r="Y13" t="n">
-        <v>0.22</v>
+        <v>0</v>
       </c>
       <c r="Z13" t="n">
-        <v>76.3</v>
+        <v>1</v>
       </c>
       <c r="AA13" t="n">
-        <v>445.2</v>
+        <v>0</v>
       </c>
       <c r="AB13" t="n">
         <v>0</v>
@@ -1973,7 +1917,7 @@
         <v>0</v>
       </c>
       <c r="AD13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE13" t="n">
         <v>0</v>
@@ -1982,33 +1926,20 @@
         <v>0</v>
       </c>
       <c r="AG13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AH13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI13" t="n">
         <v>0</v>
       </c>
-      <c r="AJ13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK13" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL13" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM13" t="n">
-        <v>144</v>
-      </c>
-      <c r="AN13" t="n">
-        <v>110</v>
-      </c>
+      <c r="AJ13" t="inlineStr"/>
+      <c r="AK13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>53955359</v>
+        <v>52800188</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -2016,74 +1947,88 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>83.6714579055441</v>
-      </c>
-      <c r="D14" t="inlineStr"/>
+        <v>93.68104038329911</v>
+      </c>
+      <c r="D14" t="n">
+        <v>23.4256055363322</v>
+      </c>
       <c r="E14" t="n">
-        <v>19.8791026005112</v>
-      </c>
-      <c r="F14" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>60</v>
+      </c>
       <c r="G14" t="n">
         <v>1</v>
       </c>
       <c r="H14" t="n">
-        <v>55</v>
-      </c>
-      <c r="I14" t="inlineStr"/>
+        <v>283</v>
+      </c>
+      <c r="I14" t="n">
+        <v>130</v>
+      </c>
       <c r="J14" t="n">
-        <v>0</v>
-      </c>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
+        <v>112</v>
+      </c>
+      <c r="K14" t="n">
+        <v>525</v>
+      </c>
+      <c r="L14" t="n">
+        <v>247</v>
+      </c>
+      <c r="M14" t="n">
+        <v>130</v>
+      </c>
+      <c r="N14" t="n">
+        <v>102</v>
+      </c>
       <c r="O14" t="n">
-        <v>126</v>
+        <v>479</v>
       </c>
       <c r="P14" t="n">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="Q14" t="n">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="R14" t="n">
-        <v>258</v>
+        <v>0</v>
       </c>
       <c r="S14" t="n">
-        <v>115</v>
+        <v>49</v>
       </c>
       <c r="T14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U14" t="n">
-        <v>20</v>
+        <v>26.8</v>
       </c>
       <c r="V14" t="n">
-        <v>135</v>
+        <v>0.17</v>
       </c>
       <c r="W14" t="n">
-        <v>2</v>
+        <v>27.02450933700383</v>
       </c>
       <c r="X14" t="n">
-        <v>22</v>
+        <v>26.76424046872996</v>
       </c>
       <c r="Y14" t="n">
-        <v>0.22</v>
+        <v>0</v>
       </c>
       <c r="Z14" t="n">
-        <v>70.40000000000001</v>
+        <v>1</v>
       </c>
       <c r="AA14" t="n">
-        <v>377.7</v>
+        <v>0</v>
       </c>
       <c r="AB14" t="n">
         <v>0</v>
       </c>
       <c r="AC14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AE14" t="n">
         <v>0</v>
@@ -2095,30 +2040,17 @@
         <v>0</v>
       </c>
       <c r="AH14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI14" t="n">
-        <v>1</v>
-      </c>
-      <c r="AJ14" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK14" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL14" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM14" t="n">
-        <v>140</v>
-      </c>
-      <c r="AN14" t="n">
-        <v>150</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AJ14" t="inlineStr"/>
+      <c r="AK14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>55642168</v>
+        <v>55333786</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -2126,65 +2058,71 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>82.4695414099932</v>
-      </c>
-      <c r="D15" t="inlineStr"/>
+        <v>86.7433264887064</v>
+      </c>
+      <c r="D15" t="n">
+        <v>19.0311418685121</v>
+      </c>
       <c r="E15" t="n">
-        <v>24.5778671518401</v>
-      </c>
-      <c r="F15" t="inlineStr"/>
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>52</v>
+      </c>
       <c r="G15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" t="n">
-        <v>55</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
-      <c r="J15" t="n">
-        <v>1</v>
-      </c>
+      <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
+      <c r="L15" t="n">
+        <v>341</v>
+      </c>
+      <c r="M15" t="n">
+        <v>320</v>
+      </c>
+      <c r="N15" t="n">
+        <v>374</v>
+      </c>
       <c r="O15" t="n">
-        <v>435.7692</v>
+        <v>1035</v>
       </c>
       <c r="P15" t="n">
-        <v>471.15186</v>
+        <v>0</v>
       </c>
       <c r="Q15" t="n">
-        <v>348.57095</v>
+        <v>7</v>
       </c>
       <c r="R15" t="n">
-        <v>1255.492</v>
+        <v>161</v>
       </c>
       <c r="S15" t="n">
-        <v>51</v>
+        <v>168</v>
       </c>
       <c r="T15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U15" t="n">
-        <v>175</v>
+        <v>22.8</v>
       </c>
       <c r="V15" t="n">
-        <v>226</v>
+        <v>0.33</v>
       </c>
       <c r="W15" t="n">
-        <v>1</v>
+        <v>27.34281922318762</v>
       </c>
       <c r="X15" t="n">
-        <v>27.29889</v>
+        <v>23.64216910815792</v>
       </c>
       <c r="Y15" t="n">
-        <v>0.22</v>
+        <v>0</v>
       </c>
       <c r="Z15" t="n">
-        <v>86.90398999999999</v>
+        <v>0</v>
       </c>
       <c r="AA15" t="n">
-        <v>573.0519</v>
+        <v>1</v>
       </c>
       <c r="AB15" t="n">
         <v>0</v>
@@ -2205,25 +2143,16 @@
         <v>0</v>
       </c>
       <c r="AH15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AI15" t="n">
         <v>0</v>
       </c>
       <c r="AJ15" t="n">
-        <v>0</v>
+        <v>148</v>
       </c>
       <c r="AK15" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL15" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM15" t="n">
-        <v>148</v>
-      </c>
-      <c r="AN15" t="n">
-        <v>137</v>
+        <v>131</v>
       </c>
     </row>
   </sheetData>

</xml_diff>